<commit_message>
Clarify present value heading in exercise 3.2
</commit_message>
<xml_diff>
--- a/outputs/01a15558-33a2-7ab0-8172-87a04b40c77e/kapitel-03-beregninger.xlsx
+++ b/outputs/01a15558-33a2-7ab0-8172-87a04b40c77e/kapitel-03-beregninger.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.1" sheetId="1" r:id="Ra87863739b8f476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.2" sheetId="2" r:id="R0a8cd77b5b1743f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.3" sheetId="3" r:id="R02fec65bb00d40fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.4" sheetId="4" r:id="R9dd4044312a147a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.5" sheetId="5" r:id="R5b1ca6aec18844d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.6" sheetId="6" r:id="R97660ddbf38d4b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.1" sheetId="1" r:id="R3330d10b13734829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.2" sheetId="2" r:id="Rcf36d33a828c462e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.3" sheetId="3" r:id="R59e12632c6c447dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.4" sheetId="4" r:id="R7c6faae64b9b4b03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.5" sheetId="5" r:id="R35725f3f70e0494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.6" sheetId="6" r:id="Rc7cab167aa7b4977"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1302,7 +1302,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb99a32c1bdb84b50"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e4f744741de4c87"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1337,7 +1337,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R192fb3fea060445e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba30c0a184ce4d27"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1372,7 +1372,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2fdaed335a9844ff"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd7b8b2d3c66f4f66"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1407,7 +1407,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R966e8afd70384187"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08171322637a4e65"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1442,7 +1442,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R410f285df78c47db"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R28af739d28af48f4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2372,7 +2372,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36a78f55461b4cf2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6e056fbc5a34c44"/>
 </x:worksheet>
 </file>
 
@@ -2639,7 +2639,7 @@
         <x:v>PV af tidlige kuponer</x:v>
       </x:c>
       <x:c r="E18" s="20" t="str">
-        <x:v>Pris til slutbetaling</x:v>
+        <x:v>Nutidsværdi af slutbetalingen</x:v>
       </x:c>
       <x:c r="F18" s="20" t="str">
         <x:v>Slutbetaling</x:v>
@@ -3320,7 +3320,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15e9b54656bf485c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fde3eccb8a2459c"/>
 </x:worksheet>
 </file>
 
@@ -4055,7 +4055,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbba1667135fe4b96"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b36f2b3ac084b47"/>
 </x:worksheet>
 </file>
 
@@ -4630,7 +4630,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7011908e3e34f19"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3eb2641d22e4462"/>
 </x:worksheet>
 </file>
 
@@ -6116,6 +6116,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ca74cc655484fd4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbb3df7afce54986"/>
 </x:worksheet>
 </file>
</xml_diff>